<commit_message>
implementado archivo de cuentos
</commit_message>
<xml_diff>
--- a/actions/corpus/cuentos.xlsx
+++ b/actions/corpus/cuentos.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,13 +29,19 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="003b4a24"/>
       <sz val="14"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="003b4a24"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +52,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="003b4a24"/>
         <bgColor rgb="003b4a24"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fff8e1"/>
+        <bgColor rgb="00fff8e1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e8f5e9"/>
+        <bgColor rgb="00e8f5e9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fff3e0"/>
+        <bgColor rgb="00fff3e0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f3e5f5"/>
+        <bgColor rgb="00f3e5f5"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,15 +91,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,16 +475,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -484,18 +524,18 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="80" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>pescador_shipibo</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>El pescador shipibo</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -508,7 +548,7 @@
           <t>En este fragmento aparece el río. ¿Cómo se dice 'agua' en shipibo?</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>jene</t>
         </is>
@@ -519,18 +559,18 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="80" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>pescador_shipibo</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>El pescador shipibo</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -543,7 +583,7 @@
           <t>¿Cómo se dice 'pez' en shipibo?</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>waka</t>
         </is>
@@ -554,18 +594,18 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>pescador_shipibo</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>El pescador shipibo</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -578,7 +618,7 @@
           <t>Ronin usa sus manos para soltar al pez. ¿Cómo se dice 'mano' en shipibo?</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>meno</t>
         </is>
@@ -589,18 +629,18 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>pescador_shipibo</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>El pescador shipibo</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="2" t="n">
         <v>4</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -609,8 +649,439 @@
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>motelo_tigre</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>El motelo y el tigre</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Un día, el tigre salió muy hambriento a buscar comida por el bosque. 🐆 Caminaba con paso firme, mirando entre los árboles.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>El tigre es el felino más grande de la Amazonía. ¿Cómo se dice 'jaguar' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>ino</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>El felino más grande y respetado de la Amazonía se llama 'ino' en shipibo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>motelo_tigre</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>El motelo y el tigre</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>En el camino, el tigre se encontró con un motelo, una pequeña tortuga de tierra. 🐢 Lo miró con ojos hambrientos y dijo: '¡Te voy a comer!'</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>El motelo es una tortuga. ¿Cómo se dice 'tortuga' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>shahue</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>El motelo tiene caparazón duro y se llama 'shahue' en shipibo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>motelo_tigre</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>El motelo y el tigre</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>El motelo, muy astuto, le respondió: 'Antes de comerme, midamos nuestras fuerzas. Atemos nuestros pies con una soga y jalemos cada uno hacia un lado.' El tigre aceptó.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Para la prueba ataron sus pies. ¿Cómo se dice 'pie' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>tae</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>La parte del cuerpo con la que caminamos se dice 'tae' en shipibo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="80" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>motelo_tigre</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>El motelo y el tigre</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>El motelo se metió al agua y, en secreto, ató la soga a una vaca marina dormida. Luego se escondió entre las hierbas para observar.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>El motelo se metió al agua. ¿Cómo se dice 'agua' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>jene</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>El motelo se metió al 'jene' (agua) para esconder su truco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="80" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>motelo_tigre</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>El motelo y el tigre</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>La vaca marina jaló con tanta fuerza que el tigre cayó vencido. Así, con su inteligencia, el motelo demostró que el más pequeño también puede ganar. 🌿</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="80" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>paujil_fiesta</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>El paujil en la fiesta</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>El paujil es un ave hermosa de la selva amazónica. 🦃 Caminaba siempre solo, pero un día se aburrió y decidió buscar diversión.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>El paujil es un ave de la selva. ¿Cómo se dice 'ave' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>isa</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Los animales que tienen plumas y vuelan se llaman 'isa' en shipibo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>paujil_fiesta</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>El paujil en la fiesta</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Mientras caminaba, escuchó música a lo lejos: ¡era una fiesta! Llegó y vio al mono tocando el tambor con mucha alegría. 🐒</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>El mono tocaba el tambor. ¿Cómo se dice 'mono' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>hiso</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>El animal que trepa los árboles con agilidad se llama 'hiso' en shipibo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>paujil_fiesta</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>El paujil en la fiesta</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Todos los animales bailaban. El paujil, que es del tamaño de una gallina, se animó y aceptó bailar también. 🎉</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>El paujil es del tamaño de una gallina. ¿Cómo se dice 'gallina' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>atapa</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>El ave de corral que pone huevos se llama 'atapa' en shipibo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>paujil_fiesta</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>El paujil en la fiesta</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Mientras bailaba, se resbaló y se manchó la cola con masato. Por eso, hasta hoy, el paujil tiene plumas de color blanco en su cola. 🪶</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Sus plumas quedaron blancas. ¿Cómo se dice 'blanco' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>josho</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>El color de las nubes y la leche se dice 'josho' en shipibo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>matrimonio_shipibo</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>El matrimonio shipibo</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>En la cultura shipibo, el matrimonio era una decisión muy importante. 🏡 El padre de la joven buscaba un hombre capaz de mantener bien la casa de su futura familia.</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>El joven debía mantener bien la casa. ¿Cómo se dice 'casa' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>shobo</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>El lugar donde vive la familia shipibo se llama 'shobo'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="80" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>matrimonio_shipibo</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>El matrimonio shipibo</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Cuando un joven pedía la mano de la chica, el suegro le hacía dos pruebas. Primero, le tocaba las palmas de las manos para sentir si era trabajador.</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Le tocaba las palmas de las manos. ¿Cómo se dice 'mano' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>meno</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>La parte del cuerpo con la que trabajamos y agarramos se dice 'meno'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="80" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>matrimonio_shipibo</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>El matrimonio shipibo</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>La segunda prueba era más difícil: el joven tenía que tumbar un árbol grande de shihuahuaco con su hacha. 🌳 Solo así demostraba su fuerza.</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Tenía que tumbar un árbol. ¿Cómo se dice 'árbol' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>jihui</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Lo que crece alto en la selva con tronco y hojas se llama 'jihui'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="80" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>matrimonio_shipibo</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>El matrimonio shipibo</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Si el joven pasaba las dos pruebas, podía casarse con su amada. Después de la boda, era el suegro quien iba a vivir a la casa del yerno. 🌿 Así eran las costumbres shipibo.</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -623,16 +1094,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Formato del corpus de cuentos</t>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Corpus de cuentos interactivos — Pishico Bot</t>
         </is>
       </c>
     </row>
@@ -640,141 +1111,290 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Columnas:</t>
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>ESTRUCTURA DEL ARCHIVO</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  cuento_id            Identificador único en minúsculas (ej. pescador_shipibo, mujer_diseno_kene)</t>
+          <t xml:space="preserve">  Cada fila representa un fragmento de un cuento.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  cuento_titulo        Nombre legible (ej. El pescador shipibo)</t>
+          <t xml:space="preserve">  Los fragmentos de un mismo cuento comparten cuento_id y cuento_titulo.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  orden                Número del fragmento dentro del cuento (1, 2, 3, ...)</t>
+          <t xml:space="preserve">  El campo 'orden' define la secuencia (1, 2, 3, ...).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  texto                Párrafo del cuento (puede contener emojis y saltos de línea con \n)</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  pregunta             Pregunta al usuario (vacío si el fragmento no tiene pregunta)</t>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>COLUMNAS</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  respuesta_esperada   Palabra shipibo canónica esperada (vacío si no hay pregunta)</t>
+          <t xml:space="preserve">  cuento_id            Identificador único del cuento (snake_case).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ayuda                Pista pedagógica para cuando el usuario falla (vacío si no aplica)</t>
+          <t xml:space="preserve">  cuento_titulo        Nombre legible que se muestra al usuario.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  orden                Posición del fragmento dentro del cuento.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Reglas:</t>
+          <t xml:space="preserve">  texto                Texto narrativo del fragmento (puede contener emojis).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Todos los fragmentos de un cuento comparten el mismo cuento_id y cuento_titulo.</t>
+          <t xml:space="preserve">  pregunta             Pregunta pedagógica (vacío si no hay).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • El campo 'orden' define la secuencia de presentación, empezando en 1.</t>
+          <t xml:space="preserve">  respuesta_esperada   Palabra shipibo canónica (debe coincidir con palabras.xlsx).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Los últimos fragmentos suelen ser de cierre y no tienen pregunta.</t>
+          <t xml:space="preserve">  ayuda                Pista pedagógica que se da cuando el usuario falla.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Las respuestas esperadas deben usar las grafías canónicas del corpus validado</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    (ver palabras.xlsx). No usar grafías obsoletas como 'yapa' o 'meken'.</t>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>CUENTOS INCLUIDOS EN ESTA VERSIÓN</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  pescador_shipibo     — El pescador shipibo  (4 fragmentos)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Para agregar un nuevo cuento:</t>
+          <t xml:space="preserve">                         Palabras: agua (jene), pez (waka), mano (meno)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1. Validar el texto y las preguntas con el asesor lingüístico.</t>
+          <t xml:space="preserve">  motelo_tigre         — El motelo y el tigre (5 fragmentos)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2. Agregar las filas en este Excel respetando el formato.</t>
+          <t xml:space="preserve">                         Palabras: jaguar (ino), tortuga (shahue),</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. Reiniciar el Action Server (rasa run actions).</t>
+          <t xml:space="preserve">                                   pie (tae), agua (jene)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4. El nuevo cuento aparecerá automáticamente como opción para el usuario.</t>
+          <t xml:space="preserve">  paujil_fiesta        — El paujil en la fiesta (4 fragmentos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                         Palabras: ave (isa), mono (hiso),</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                   gallina (atapa), blanco (josho)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  matrimonio_shipibo   — El matrimonio shipibo (4 fragmentos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                         Palabras: casa (shobo), mano (meno), árbol (jihui)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TOTAL: 4 cuentos, 17 fragmentos, 14 preguntas pedagógicas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Cobertura: las 5 categorías del corpus se ejercitan al menos una vez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>PENDIENTES PARA EL ASESOR LINGÜÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Los textos en español son borradores libres basados en los cuentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    originales del corpus Cuentos.zip (es-shp9, es-shp4, es-shp14).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Revisar fidelidad cultural y narrativa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Las preguntas y pistas pedagógicas son redacción nueva: revisar tono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Las respuestas_esperadas usan las grafías canónicas de palabras.xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Pendiente: producir las versiones shipibo de cada fragmento para</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    soportar el modo de práctica shp→es en cuentos (a futuro).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>REGLAS PARA AGREGAR NUEVOS CUENTOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. Validar el texto con el asesor lingüístico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. Las respuestas_esperadas deben venir de palabras.xlsx (no inventar grafías).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3. El último fragmento suele ser de cierre y no tiene pregunta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4. Mantener fragmentos entre 1-3 oraciones para no saturar al usuario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5. Reiniciar el Action Server (rasa run actions) — no requiere rasa train.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
mejoras en conversa conmigo
</commit_message>
<xml_diff>
--- a/actions/corpus/cuentos.xlsx
+++ b/actions/corpus/cuentos.xlsx
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -110,6 +110,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -475,16 +478,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,564 +528,440 @@
       </c>
     </row>
     <row r="2" ht="80" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>pescador_shipibo</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>El pescador shipibo</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>motelo_tigre</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>El motelo y el tigre</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Había una vez un pescador shipibo llamado Ronin. 🛶 Cada mañana iba al río con su canoa para pescar.</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>En este fragmento aparece el río. ¿Cómo se dice 'agua' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Un día, el tigre salió muy hambriento a buscar comida por el bosque. 🐆 Caminaba con paso firme, mirando entre los árboles.</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>El tigre es el felino más grande de la Amazonía. ¿Cómo se dice 'jaguar' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>ino</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>Es el felino más grande y respetado de la Amazonía. Vive en la selva y caza al acecho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="80" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>motelo_tigre</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>El motelo y el tigre</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>En el camino, el tigre se encontró con un motelo, una pequeña tortuga de tierra. 🐢 Lo miró con ojos hambrientos y dijo: '¡Te voy a comer!'</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>El motelo es una tortuga. ¿Cómo se dice 'tortuga' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>shahue</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Animal con caparazón duro que vive en ríos y lagunas. Se mueve lento pero es muy resistente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>motelo_tigre</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>El motelo y el tigre</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>El motelo, muy astuto, le respondió: 'Antes de comerme, midamos nuestras fuerzas. Atemos nuestros pies con una soga y jalemos cada uno hacia un lado.' El tigre aceptó.</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Para la prueba ataron sus pies. ¿Cómo se dice 'pie' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>tae</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>La parte del cuerpo que tocamos con el suelo al caminar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>motelo_tigre</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>El motelo y el tigre</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>El motelo se metió al agua y, en secreto, ató la soga a una vaca marina dormida. Luego se escondió entre las hierbas para observar.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>El motelo se metió al agua. ¿Cómo se dice 'agua' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>jene</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>El río está lleno de agua. En shipibo, agua se dice 'jene'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="80" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>pescador_shipibo</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>El pescador shipibo</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Sin esto no podríamos vivir. Corre por los ríos de la Amazonía y la bebemos cada día.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>motelo_tigre</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>El motelo y el tigre</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>La vaca marina jaló con tanta fuerza que el tigre cayó vencido. Así, con su inteligencia, el motelo demostró que el más pequeño también puede ganar. 🌿</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="8" t="n"/>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>paujil_fiesta</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>El paujil en la fiesta</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>El paujil es un ave hermosa de la selva amazónica. 🦃 Caminaba siempre solo, pero un día se aburrió y decidió buscar diversión.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>El paujil es un ave de la selva. ¿Cómo se dice 'ave' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>isa</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Animal con plumas que puede volar por el cielo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>paujil_fiesta</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>El paujil en la fiesta</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Ronin pescaba muchos peces para alimentar a su familia. Un día vio un pez grande y brillante.</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>¿Cómo se dice 'pez' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>waka</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Recuerda: el animal que Ronin pesca se llama 'waka' en shipibo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>pescador_shipibo</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>El pescador shipibo</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Mientras caminaba, escuchó música a lo lejos: ¡era una fiesta! Llegó y vio al mono tocando el tambor con mucha alegría. 🐒</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>El mono tocaba el tambor. ¿Cómo se dice 'mono' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>hiso</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Trepa los árboles con mucha agilidad. Muy común en la selva amazónica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="80" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>paujil_fiesta</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>El paujil en la fiesta</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>El pez le habló a Ronin: 'Si me dejas vivir, te enseñaré las palabras antiguas de la selva.'</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Ronin usa sus manos para soltar al pez. ¿Cómo se dice 'mano' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Todos los animales bailaban. El paujil, que es del tamaño de una gallina, se animó y aceptó bailar también. 🎉</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>El paujil es del tamaño de una gallina. ¿Cómo se dice 'gallina' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>atapa</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Ave de corral que pone huevos y vive cerca de las casas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="80" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>paujil_fiesta</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>El paujil en la fiesta</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Mientras bailaba, se resbaló y se manchó la cola con masato. Por eso, hasta hoy, el paujil tiene plumas de color blanco en su cola. 🪶</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Sus plumas quedaron blancas. ¿Cómo se dice 'blanco' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>josho</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>El color de las nubes y de la leche.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="80" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>matrimonio_shipibo</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>El matrimonio shipibo</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>En la cultura shipibo, el matrimonio era una decisión muy importante. 🏡 El padre de la joven buscaba un hombre capaz de mantener bien la casa de su futura familia.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>El joven debía mantener bien la casa. ¿Cómo se dice 'casa' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>shobo</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>El lugar donde vive y se reúne una familia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>matrimonio_shipibo</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>El matrimonio shipibo</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Cuando un joven pedía la mano de la chica, el suegro le hacía dos pruebas. Primero, le tocaba las palmas de las manos para sentir si era trabajador.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Le tocaba las palmas de las manos. ¿Cómo se dice 'mano' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>meno</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>La parte del cuerpo con la que agarramos cosas se dice 'meno'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>pescador_shipibo</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>El pescador shipibo</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>La parte del cuerpo con la que escribimos, agarramos y creamos cosas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>matrimonio_shipibo</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>El matrimonio shipibo</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>La segunda prueba era más difícil: el joven tenía que tumbar un árbol grande de shihuahuaco con su hacha. 🌳 Solo así demostraba su fuerza.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Tenía que tumbar un árbol. ¿Cómo se dice 'árbol' en shipibo?</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>jihui</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Crece alto en la selva. Tiene tronco, ramas y hojas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>matrimonio_shipibo</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>El matrimonio shipibo</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Ronin aceptó. Así aprendió muchas palabras antiguas y compartió el conocimiento con su pueblo. 🌿</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>motelo_tigre</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>El motelo y el tigre</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Un día, el tigre salió muy hambriento a buscar comida por el bosque. 🐆 Caminaba con paso firme, mirando entre los árboles.</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>El tigre es el felino más grande de la Amazonía. ¿Cómo se dice 'jaguar' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>ino</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>El felino más grande y respetado de la Amazonía se llama 'ino' en shipibo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>motelo_tigre</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>El motelo y el tigre</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>En el camino, el tigre se encontró con un motelo, una pequeña tortuga de tierra. 🐢 Lo miró con ojos hambrientos y dijo: '¡Te voy a comer!'</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>El motelo es una tortuga. ¿Cómo se dice 'tortuga' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>shahue</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>El motelo tiene caparazón duro y se llama 'shahue' en shipibo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="80" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>motelo_tigre</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>El motelo y el tigre</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>El motelo, muy astuto, le respondió: 'Antes de comerme, midamos nuestras fuerzas. Atemos nuestros pies con una soga y jalemos cada uno hacia un lado.' El tigre aceptó.</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Para la prueba ataron sus pies. ¿Cómo se dice 'pie' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>tae</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>La parte del cuerpo con la que caminamos se dice 'tae' en shipibo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="80" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>motelo_tigre</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>El motelo y el tigre</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>El motelo se metió al agua y, en secreto, ató la soga a una vaca marina dormida. Luego se escondió entre las hierbas para observar.</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>El motelo se metió al agua. ¿Cómo se dice 'agua' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>jene</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>El motelo se metió al 'jene' (agua) para esconder su truco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="80" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>motelo_tigre</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>El motelo y el tigre</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>La vaca marina jaló con tanta fuerza que el tigre cayó vencido. Así, con su inteligencia, el motelo demostró que el más pequeño también puede ganar. 🌿</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="3" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11" ht="80" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>paujil_fiesta</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>El paujil en la fiesta</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>El paujil es un ave hermosa de la selva amazónica. 🦃 Caminaba siempre solo, pero un día se aburrió y decidió buscar diversión.</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>El paujil es un ave de la selva. ¿Cómo se dice 'ave' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>isa</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>Los animales que tienen plumas y vuelan se llaman 'isa' en shipibo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="80" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>paujil_fiesta</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>El paujil en la fiesta</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Mientras caminaba, escuchó música a lo lejos: ¡era una fiesta! Llegó y vio al mono tocando el tambor con mucha alegría. 🐒</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>El mono tocaba el tambor. ¿Cómo se dice 'mono' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>hiso</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>El animal que trepa los árboles con agilidad se llama 'hiso' en shipibo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="80" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>paujil_fiesta</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>El paujil en la fiesta</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Todos los animales bailaban. El paujil, que es del tamaño de una gallina, se animó y aceptó bailar también. 🎉</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>El paujil es del tamaño de una gallina. ¿Cómo se dice 'gallina' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>atapa</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>El ave de corral que pone huevos se llama 'atapa' en shipibo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="80" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>paujil_fiesta</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>El paujil en la fiesta</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Mientras bailaba, se resbaló y se manchó la cola con masato. Por eso, hasta hoy, el paujil tiene plumas de color blanco en su cola. 🪶</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Sus plumas quedaron blancas. ¿Cómo se dice 'blanco' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>josho</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>El color de las nubes y la leche se dice 'josho' en shipibo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="80" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>matrimonio_shipibo</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>El matrimonio shipibo</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>En la cultura shipibo, el matrimonio era una decisión muy importante. 🏡 El padre de la joven buscaba un hombre capaz de mantener bien la casa de su futura familia.</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>El joven debía mantener bien la casa. ¿Cómo se dice 'casa' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>shobo</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>El lugar donde vive la familia shipibo se llama 'shobo'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="80" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>matrimonio_shipibo</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>El matrimonio shipibo</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Cuando un joven pedía la mano de la chica, el suegro le hacía dos pruebas. Primero, le tocaba las palmas de las manos para sentir si era trabajador.</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Le tocaba las palmas de las manos. ¿Cómo se dice 'mano' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>meno</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>La parte del cuerpo con la que trabajamos y agarramos se dice 'meno'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="80" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>matrimonio_shipibo</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>El matrimonio shipibo</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>La segunda prueba era más difícil: el joven tenía que tumbar un árbol grande de shihuahuaco con su hacha. 🌳 Solo así demostraba su fuerza.</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Tenía que tumbar un árbol. ¿Cómo se dice 'árbol' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>jihui</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>Lo que crece alto en la selva con tronco y hojas se llama 'jihui'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="80" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>matrimonio_shipibo</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>El matrimonio shipibo</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Si el joven pasaba las dos pruebas, podía casarse con su amada. Después de la boda, era el suegro quien iba a vivir a la casa del yerno. 🌿 Así eran las costumbres shipibo.</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr"/>
-      <c r="F18" s="5" t="inlineStr"/>
-      <c r="G18" s="5" t="inlineStr"/>
-    </row>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="80" customHeight="1"/>
+    <row r="16" ht="80" customHeight="1"/>
+    <row r="17" ht="80" customHeight="1"/>
+    <row r="18" ht="80" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1107,9 +986,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1138,9 +1015,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
@@ -1197,9 +1072,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
@@ -1277,9 +1150,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
@@ -1294,9 +1165,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-    </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
@@ -1353,9 +1222,7 @@
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-    </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
voacbulario y cuentos alineados
</commit_message>
<xml_diff>
--- a/actions/corpus/cuentos.xlsx
+++ b/actions/corpus/cuentos.xlsx
@@ -590,17 +590,17 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>El anciano fue a pescar. ¿Cómo se dice 'pescar' en shipibo?</t>
+          <t>El anciano fue a la cocha. ¿Cómo se dice 'cocha' en shipibo?</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>yomerati</t>
+          <t>ian</t>
         </is>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>Es una actividad que se realiza en ríos, cochas o lagunas para obtener peces.</t>
+          <t>Es un lago o laguna donde se pesca, muy común en la Amazonía.</t>
         </is>
       </c>
     </row>
@@ -693,21 +693,9 @@
           <t>El camungo levantó vuelo y se alejó. El anciano quedó sorprendido por lo que había escuchado en la cocha. 🌿</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>El anciano estaba en la cocha. ¿Cómo se dice 'cocha' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>ian</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>Es una laguna o cuerpo de agua donde se puede pescar.</t>
-        </is>
-      </c>
+      <c r="E9" s="14" t="n"/>
+      <c r="F9" s="14" t="n"/>
+      <c r="G9" s="14" t="n"/>
     </row>
     <row r="10" ht="80" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
@@ -730,17 +718,17 @@
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>La actividad principal del cuento es pescar. ¿Cómo se dice 'pescar' en shipibo?</t>
+          <t>Los que se organizaban para pescar eran los hombres. ¿Cómo se dice 'hombre' en shipibo?</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>yomerati</t>
+          <t>joni</t>
         </is>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>Es una actividad importante para conseguir alimento en el río o la cocha.</t>
+          <t>Se refiere a una persona de sexo masculino.</t>
         </is>
       </c>
     </row>
@@ -835,17 +823,17 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Los pescadores llegaban al puerto. ¿Cómo se dice 'puerto' en shipibo?</t>
+          <t>Cuando regresaban, llegaban al puerto con sus canoas. ¿Cómo se dice 'canoa' en shipibo?</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>repinti</t>
+          <t>nonti</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>Es el lugar de llegada junto al río o la cocha.</t>
+          <t>Es una embarcación de madera para navegar por el río.</t>
         </is>
       </c>
     </row>
@@ -926,21 +914,6 @@
           <t>La joven era especial porque tenía muchos pretendientes que la querían.</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Ella tenía varios enamorados. ¿Cómo se dice 'enamorarse' en shipibo?</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>merati</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Es la acción de querer a alguien de manera especial.</t>
-        </is>
-      </c>
     </row>
     <row r="17" ht="80" customHeight="1">
       <c r="A17" t="inlineStr">
@@ -1033,17 +1006,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>El ave quedó con una marca especial. ¿Cómo se dice 'rayas' en shipibo?</t>
+          <t>El shihuango es un tipo de ave. ¿Cómo se dice 'ave' en shipibo?</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>chisereya</t>
+          <t>isa</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Son líneas o marcas que se ven sobre el cuerpo de un animal.</t>
+          <t>Es un animal con plumas que puede volar.</t>
         </is>
       </c>
     </row>
@@ -1079,9 +1052,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1131,9 +1101,6 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -1176,9 +1143,6 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -1235,9 +1199,6 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
@@ -1273,9 +1234,6 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr"/>
-    </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
@@ -1395,9 +1353,6 @@
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-    </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
@@ -1412,9 +1367,6 @@
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-    </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
@@ -1492,9 +1444,6 @@
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="inlineStr"/>
-    </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
@@ -1515,9 +1464,6 @@
           <t xml:space="preserve">  es-shp13 es valioso culturalmente, pero funciona mejor como módulo de cultura/costumbres.</t>
         </is>
       </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1701,7 +1647,6 @@
           <t>Sirve para señalar el lugar donde estamos o donde ocurre algo.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1737,7 +1682,6 @@
           <t>Es una acción: sujetar algo con una cuerda, soga o lazo.</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1773,7 +1717,6 @@
           <t>Es una acción: tirar algo hacia uno mismo o hacia un lado.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1794,7 +1737,6 @@
           <t>Al final, el tigre terminó cansado y el motelo demostró que la inteligencia también puede vencer a la fuerza. 🌿</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1870,7 +1812,6 @@
           <t>Es una actividad relacionada con el río y la alimentación.</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1906,7 +1847,6 @@
           <t>Se relaciona con formar un hogar y preparar un lugar para vivir.</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1942,7 +1882,6 @@
           <t>Es una acción: derribar algo, como un árbol, usando fuerza o herramienta.</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1963,7 +1902,6 @@
           <t>Si el joven superaba las pruebas, podía casarse. Luego, según la costumbre, el suegro podía vivir en la casa del yerno. 🌿</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>